<commit_message>
Filtros por defecto y orden cronologico ajustado
</commit_message>
<xml_diff>
--- a/datos/marvel_db.xlsx
+++ b/datos/marvel_db.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elena\Documents\ELENA\marvel_list\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9961DC61-16E3-438C-9A4A-C72799F8AABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D9E91D3-C8EF-4234-B4EE-DD2493CF13AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-21713" yWindow="-113" windowWidth="21826" windowHeight="13006" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="88">
   <si>
     <t>id_tmdb</t>
   </si>
@@ -256,9 +256,6 @@
     <t>Daredevil</t>
   </si>
   <si>
-    <t>Defenders / MCU</t>
-  </si>
-  <si>
     <t>Saga Defenders</t>
   </si>
   <si>
@@ -280,10 +277,13 @@
     <t>Agentes de S.H.I.E.L.D.</t>
   </si>
   <si>
-    <t>Marvel Television</t>
-  </si>
-  <si>
     <t>Agent Carter</t>
+  </si>
+  <si>
+    <t>Spider-Man: Brand New Day</t>
+  </si>
+  <si>
+    <t>MCU / Defenders</t>
   </si>
 </sst>
 </file>
@@ -655,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="30.6328125" bestFit="1" customWidth="1"/>
@@ -689,293 +689,326 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>36657</v>
+        <v>1771</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>100</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>36658</v>
+        <v>61550</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E3">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>36668</v>
+        <v>299537</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E4">
-        <v>30</v>
+        <v>150</v>
+      </c>
+      <c r="F4">
+        <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>2080</v>
+        <v>1726</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>200</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>49538</v>
+        <v>1724</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E6">
+        <v>300</v>
+      </c>
+      <c r="F6">
         <v>1</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>76170</v>
+        <v>10138</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>40</v>
+        <v>350</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>127585</v>
+        <v>10195</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E8">
-        <v>50</v>
+        <v>400</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>293660</v>
+        <v>24428</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E9">
-        <v>70</v>
+        <v>500</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>246655</v>
+        <v>1403</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E10">
-        <v>15</v>
+        <v>510</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>263115</v>
+        <v>68721</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E11">
-        <v>90</v>
+        <v>520</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>383498</v>
+        <v>76338</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E12">
-        <v>80</v>
+        <v>540</v>
+      </c>
+      <c r="F12">
+        <v>2</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>320288</v>
+        <v>100402</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E13">
-        <v>25</v>
+        <v>560</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>340102</v>
+        <v>118340</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E14">
-        <v>85</v>
+        <v>580</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
       </c>
       <c r="G14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>533535</v>
+        <v>283995</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="E15">
-        <v>860</v>
+        <v>590</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>1771</v>
+        <v>99861</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
@@ -984,10 +1017,10 @@
         <v>9</v>
       </c>
       <c r="E16">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" t="s">
         <v>10</v>
@@ -995,56 +1028,50 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>1726</v>
+        <v>61889</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D17" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E17">
-        <v>200</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
+        <v>610</v>
       </c>
       <c r="G17" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18">
-        <v>1724</v>
+        <v>38472</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D18" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E18">
-        <v>300</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
+        <v>615</v>
       </c>
       <c r="G18" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19">
-        <v>10138</v>
+        <v>102899</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
@@ -1053,10 +1080,10 @@
         <v>9</v>
       </c>
       <c r="E19">
-        <v>350</v>
+        <v>620</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="s">
         <v>10</v>
@@ -1064,56 +1091,50 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20">
-        <v>10195</v>
+        <v>62126</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D20" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E20">
-        <v>400</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
+        <v>630</v>
       </c>
       <c r="G20" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21">
-        <v>24428</v>
+        <v>62127</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E21">
-        <v>500</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
+        <v>635</v>
       </c>
       <c r="G21" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22">
-        <v>68721</v>
+        <v>271110</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1122,10 +1143,10 @@
         <v>9</v>
       </c>
       <c r="E22">
-        <v>520</v>
+        <v>640</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G22" t="s">
         <v>10</v>
@@ -1133,33 +1154,30 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23">
-        <v>76338</v>
+        <v>62285</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D23" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E23">
-        <v>540</v>
-      </c>
-      <c r="F23">
-        <v>2</v>
+        <v>645</v>
       </c>
       <c r="G23" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24">
-        <v>100402</v>
+        <v>497698</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
@@ -1168,21 +1186,21 @@
         <v>9</v>
       </c>
       <c r="E24">
-        <v>560</v>
+        <v>650</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G24" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>118340</v>
+        <v>315635</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="C25" t="s">
         <v>8</v>
@@ -1191,10 +1209,10 @@
         <v>9</v>
       </c>
       <c r="E25">
-        <v>580</v>
+        <v>660</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" t="s">
         <v>10</v>
@@ -1202,33 +1220,30 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>283995</v>
+        <v>67178</v>
       </c>
       <c r="B26" t="s">
-        <v>37</v>
+        <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>87</v>
       </c>
       <c r="E26">
-        <v>590</v>
-      </c>
-      <c r="F26">
-        <v>3</v>
+        <v>665</v>
       </c>
       <c r="G26" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>99861</v>
+        <v>284052</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="C27" t="s">
         <v>8</v>
@@ -1237,10 +1252,10 @@
         <v>9</v>
       </c>
       <c r="E27">
-        <v>600</v>
+        <v>670</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27" t="s">
         <v>10</v>
@@ -1248,10 +1263,10 @@
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>102899</v>
+        <v>284053</v>
       </c>
       <c r="B28" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C28" t="s">
         <v>8</v>
@@ -1260,10 +1275,10 @@
         <v>9</v>
       </c>
       <c r="E28">
-        <v>620</v>
+        <v>680</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28" t="s">
         <v>10</v>
@@ -1271,10 +1286,10 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29">
-        <v>271110</v>
+        <v>284054</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
@@ -1283,7 +1298,7 @@
         <v>9</v>
       </c>
       <c r="E29">
-        <v>640</v>
+        <v>690</v>
       </c>
       <c r="F29">
         <v>3</v>
@@ -1294,10 +1309,10 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>497698</v>
+        <v>299536</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C30" t="s">
         <v>8</v>
@@ -1306,21 +1321,21 @@
         <v>9</v>
       </c>
       <c r="E30">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="F30">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G30" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>315635</v>
+        <v>363088</v>
       </c>
       <c r="B31" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
@@ -1329,7 +1344,7 @@
         <v>9</v>
       </c>
       <c r="E31">
-        <v>660</v>
+        <v>710</v>
       </c>
       <c r="F31">
         <v>3</v>
@@ -1340,10 +1355,10 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>284052</v>
+        <v>299534</v>
       </c>
       <c r="B32" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C32" t="s">
         <v>8</v>
@@ -1352,7 +1367,7 @@
         <v>9</v>
       </c>
       <c r="E32">
-        <v>670</v>
+        <v>720</v>
       </c>
       <c r="F32">
         <v>3</v>
@@ -1363,56 +1378,56 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33">
-        <v>284053</v>
+        <v>84958</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="C33" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
         <v>9</v>
       </c>
       <c r="E33">
-        <v>680</v>
+        <v>725</v>
       </c>
       <c r="F33">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G33" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>284054</v>
+        <v>85271</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D34" t="s">
         <v>9</v>
       </c>
       <c r="E34">
-        <v>690</v>
+        <v>730</v>
       </c>
       <c r="F34">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G34" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>299536</v>
+        <v>429617</v>
       </c>
       <c r="B35" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C35" t="s">
         <v>8</v>
@@ -1421,7 +1436,7 @@
         <v>9</v>
       </c>
       <c r="E35">
-        <v>700</v>
+        <v>740</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -1432,33 +1447,33 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>363088</v>
+        <v>88396</v>
       </c>
       <c r="B36" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="C36" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D36" t="s">
         <v>9</v>
       </c>
       <c r="E36">
-        <v>710</v>
+        <v>745</v>
       </c>
       <c r="F36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G36" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>299537</v>
+        <v>566525</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C37" t="s">
         <v>8</v>
@@ -1467,21 +1482,21 @@
         <v>9</v>
       </c>
       <c r="E37">
-        <v>150</v>
+        <v>750</v>
       </c>
       <c r="F37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>299534</v>
+        <v>524434</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C38" t="s">
         <v>8</v>
@@ -1490,21 +1505,21 @@
         <v>9</v>
       </c>
       <c r="E38">
-        <v>720</v>
+        <v>760</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>429617</v>
+        <v>634649</v>
       </c>
       <c r="B39" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C39" t="s">
         <v>8</v>
@@ -1513,30 +1528,30 @@
         <v>9</v>
       </c>
       <c r="E39">
-        <v>740</v>
+        <v>770</v>
       </c>
       <c r="F39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G39" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40">
-        <v>566525</v>
+        <v>88329</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D40" t="s">
         <v>9</v>
       </c>
       <c r="E40">
-        <v>750</v>
+        <v>775</v>
       </c>
       <c r="F40">
         <v>4</v>
@@ -1547,10 +1562,10 @@
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41">
-        <v>524434</v>
+        <v>453395</v>
       </c>
       <c r="B41" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C41" t="s">
         <v>8</v>
@@ -1559,7 +1574,7 @@
         <v>9</v>
       </c>
       <c r="E41">
-        <v>760</v>
+        <v>780</v>
       </c>
       <c r="F41">
         <v>4</v>
@@ -1570,19 +1585,19 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42">
-        <v>634649</v>
+        <v>92749</v>
       </c>
       <c r="B42" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="C42" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D42" t="s">
         <v>9</v>
       </c>
       <c r="E42">
-        <v>770</v>
+        <v>785</v>
       </c>
       <c r="F42">
         <v>4</v>
@@ -1593,10 +1608,10 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>453395</v>
+        <v>616037</v>
       </c>
       <c r="B43" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C43" t="s">
         <v>8</v>
@@ -1605,7 +1620,7 @@
         <v>9</v>
       </c>
       <c r="E43">
-        <v>780</v>
+        <v>790</v>
       </c>
       <c r="F43">
         <v>4</v>
@@ -1616,19 +1631,19 @@
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44">
-        <v>616037</v>
+        <v>92782</v>
       </c>
       <c r="B44" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="C44" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D44" t="s">
         <v>9</v>
       </c>
       <c r="E44">
-        <v>790</v>
+        <v>795</v>
       </c>
       <c r="F44">
         <v>4</v>
@@ -1662,22 +1677,22 @@
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46">
-        <v>640146</v>
+        <v>92783</v>
       </c>
       <c r="B46" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D46" t="s">
         <v>9</v>
       </c>
       <c r="E46">
-        <v>820</v>
+        <v>805</v>
       </c>
       <c r="F46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G46" t="s">
         <v>30</v>
@@ -1685,10 +1700,10 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47">
-        <v>447365</v>
+        <v>640146</v>
       </c>
       <c r="B47" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C47" t="s">
         <v>8</v>
@@ -1697,7 +1712,7 @@
         <v>9</v>
       </c>
       <c r="E47">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="F47">
         <v>5</v>
@@ -1708,10 +1723,10 @@
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48">
-        <v>609681</v>
+        <v>447365</v>
       </c>
       <c r="B48" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
@@ -1720,7 +1735,7 @@
         <v>9</v>
       </c>
       <c r="E48">
-        <v>840</v>
+        <v>830</v>
       </c>
       <c r="F48">
         <v>5</v>
@@ -1731,19 +1746,19 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49">
-        <v>822119</v>
+        <v>114472</v>
       </c>
       <c r="B49" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="C49" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D49" t="s">
         <v>9</v>
       </c>
       <c r="E49">
-        <v>870</v>
+        <v>835</v>
       </c>
       <c r="F49">
         <v>5</v>
@@ -1754,10 +1769,10 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50">
-        <v>986056</v>
+        <v>609681</v>
       </c>
       <c r="B50" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C50" t="s">
         <v>8</v>
@@ -1766,7 +1781,7 @@
         <v>9</v>
       </c>
       <c r="E50">
-        <v>880</v>
+        <v>840</v>
       </c>
       <c r="F50">
         <v>5</v>
@@ -1777,22 +1792,22 @@
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51">
-        <v>617126</v>
+        <v>122226</v>
       </c>
       <c r="B51" t="s">
-        <v>62</v>
+        <v>74</v>
       </c>
       <c r="C51" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D51" t="s">
         <v>9</v>
       </c>
       <c r="E51">
-        <v>900</v>
+        <v>845</v>
       </c>
       <c r="F51">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G51" t="s">
         <v>30</v>
@@ -1800,22 +1815,22 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52">
-        <v>1003596</v>
+        <v>138501</v>
       </c>
       <c r="B52" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C52" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D52" t="s">
         <v>9</v>
       </c>
       <c r="E52">
-        <v>920</v>
+        <v>855</v>
       </c>
       <c r="F52">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G52" t="s">
         <v>30</v>
@@ -1823,22 +1838,22 @@
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53">
-        <v>1003598</v>
+        <v>533535</v>
       </c>
       <c r="B53" t="s">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="C53" t="s">
         <v>8</v>
       </c>
       <c r="D53" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E53">
-        <v>930</v>
+        <v>1150</v>
       </c>
       <c r="F53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G53" t="s">
         <v>30</v>
@@ -1846,10 +1861,10 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54">
-        <v>85271</v>
+        <v>202555</v>
       </c>
       <c r="B54" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="C54" t="s">
         <v>66</v>
@@ -1858,10 +1873,10 @@
         <v>9</v>
       </c>
       <c r="E54">
-        <v>730</v>
+        <v>865</v>
       </c>
       <c r="F54">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G54" t="s">
         <v>30</v>
@@ -1869,22 +1884,22 @@
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55">
-        <v>88396</v>
+        <v>822119</v>
       </c>
       <c r="B55" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C55" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D55" t="s">
         <v>9</v>
       </c>
       <c r="E55">
-        <v>745</v>
+        <v>870</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G55" t="s">
         <v>30</v>
@@ -1892,22 +1907,22 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56">
-        <v>84958</v>
+        <v>986056</v>
       </c>
       <c r="B56" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C56" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D56" t="s">
         <v>9</v>
       </c>
       <c r="E56">
-        <v>725</v>
+        <v>880</v>
       </c>
       <c r="F56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G56" t="s">
         <v>30</v>
@@ -1915,22 +1930,22 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57">
-        <v>88329</v>
+        <v>617126</v>
       </c>
       <c r="B57" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C57" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D57" t="s">
         <v>9</v>
       </c>
       <c r="E57">
-        <v>775</v>
+        <v>900</v>
       </c>
       <c r="F57">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G57" t="s">
         <v>30</v>
@@ -1938,22 +1953,22 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58">
-        <v>92749</v>
+        <v>969681</v>
       </c>
       <c r="B58" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="C58" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D58" t="s">
         <v>9</v>
       </c>
       <c r="E58">
-        <v>785</v>
+        <v>901</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G58" t="s">
         <v>30</v>
@@ -1961,22 +1976,22 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59">
-        <v>92782</v>
+        <v>1003596</v>
       </c>
       <c r="B59" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="C59" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D59" t="s">
         <v>9</v>
       </c>
       <c r="E59">
-        <v>795</v>
+        <v>920</v>
       </c>
       <c r="F59">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G59" t="s">
         <v>30</v>
@@ -1984,22 +1999,22 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>92783</v>
+        <v>1003598</v>
       </c>
       <c r="B60" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C60" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D60" t="s">
         <v>9</v>
       </c>
       <c r="E60">
-        <v>805</v>
+        <v>930</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G60" t="s">
         <v>30</v>
@@ -2007,248 +2022,262 @@
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61">
-        <v>114472</v>
+        <v>49538</v>
       </c>
       <c r="B61" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="C61" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D61" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E61">
-        <v>835</v>
-      </c>
-      <c r="F61">
-        <v>5</v>
+        <v>1010</v>
       </c>
       <c r="G61" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62">
-        <v>122226</v>
+        <v>127585</v>
       </c>
       <c r="B62" t="s">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="C62" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D62" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E62">
-        <v>845</v>
-      </c>
-      <c r="F62">
-        <v>5</v>
+        <v>1020</v>
       </c>
       <c r="G62" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>138501</v>
+        <v>2080</v>
       </c>
       <c r="B63" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="C63" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E63">
-        <v>855</v>
-      </c>
-      <c r="F63">
-        <v>5</v>
+        <v>1030</v>
       </c>
       <c r="G63" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64">
-        <v>202555</v>
+        <v>246655</v>
       </c>
       <c r="B64" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="C64" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D64" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E64">
-        <v>865</v>
-      </c>
-      <c r="F64">
-        <v>5</v>
+        <v>1040</v>
       </c>
       <c r="G64" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65">
-        <v>61889</v>
+        <v>320288</v>
       </c>
       <c r="B65" t="s">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D65" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E65">
-        <v>610</v>
+        <v>1050</v>
       </c>
       <c r="G65" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66">
-        <v>38472</v>
+        <v>36657</v>
       </c>
       <c r="B66" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="C66" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D66" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E66">
-        <v>615</v>
+        <v>1060</v>
       </c>
       <c r="G66" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67">
-        <v>62126</v>
+        <v>36658</v>
       </c>
       <c r="B67" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D67" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E67">
-        <v>630</v>
+        <v>1070</v>
       </c>
       <c r="G67" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68">
-        <v>62127</v>
+        <v>36668</v>
       </c>
       <c r="B68" t="s">
-        <v>82</v>
+        <v>17</v>
       </c>
       <c r="C68" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D68" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E68">
-        <v>635</v>
+        <v>1080</v>
       </c>
       <c r="G68" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69">
-        <v>62285</v>
+        <v>76170</v>
       </c>
       <c r="B69" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="C69" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D69" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E69">
-        <v>645</v>
+        <v>1090</v>
       </c>
       <c r="G69" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A70">
-        <v>67178</v>
+        <v>293660</v>
       </c>
       <c r="B70" t="s">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="C70" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D70" t="s">
-        <v>78</v>
+        <v>14</v>
       </c>
       <c r="E70">
-        <v>665</v>
+        <v>1100</v>
       </c>
       <c r="G70" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A71">
-        <v>1403</v>
+        <v>383498</v>
       </c>
       <c r="B71" t="s">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="C71" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D71" t="s">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E71">
-        <v>510</v>
+        <v>1110</v>
+      </c>
+      <c r="G71" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A72">
-        <v>61550</v>
+        <v>340102</v>
       </c>
       <c r="B72" t="s">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="C72" t="s">
-        <v>66</v>
+        <v>8</v>
       </c>
       <c r="D72" t="s">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="E72">
-        <v>110</v>
+        <v>1120</v>
+      </c>
+      <c r="G72" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>263115</v>
+      </c>
+      <c r="B73" t="s">
+        <v>24</v>
+      </c>
+      <c r="C73" t="s">
+        <v>8</v>
+      </c>
+      <c r="D73" t="s">
+        <v>14</v>
+      </c>
+      <c r="E73">
+        <v>1140</v>
+      </c>
+      <c r="G73" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>